<commit_message>
Publish 11-case results gallery and full 790-frame DXY-MID release validation
</commit_message>
<xml_diff>
--- a/mainline/tables/group_results.xlsx
+++ b/mainline/tables/group_results.xlsx
@@ -3575,7 +3575,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>unstable_frames</t>
+          <t>非Strict帧数</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>strict_only</t>
+          <t>是否仅Strict诊断</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -8084,82 +8084,82 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>mainline_id</t>
+          <t>正式主线</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>target_groups</t>
+          <t>目标组数</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>valid_groups</t>
+          <t>数值有效组数</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>input_frames</t>
+          <t>总输入帧数</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>valid_frames</t>
+          <t>总有效帧数</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ring_failed_frames</t>
+          <t>总Ring失败帧数</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>normal_frames</t>
+          <t>总Normal帧数</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Q_recovery_frames</t>
+          <t>总Q恢复帧数</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>strict_frames</t>
+          <t>总Strict帧数</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>median_absolute_relative_error_pct</t>
+          <t>中位绝对相对误差（%）</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>MAE_mm</t>
+          <t>MAE（mm）</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>p95_absolute_relative_error_pct</t>
+          <t>P95绝对相对误差（%）</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>max_absolute_relative_error_pct</t>
+          <t>最大绝对相对误差（%）</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>within_10pct_count</t>
+          <t>误差10%以内组数</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>within_10pct_percent</t>
+          <t>误差10%以内比例（%）</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>n_videos</t>
+          <t>总视频数</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -8169,17 +8169,17 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>threshold10_misclassified</t>
+          <t>10mm误分类组数</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>historical_prediction_fallback</t>
+          <t>历史预测回退</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>GT_used_for_algorithm_selection</t>
+          <t>是否用GT选择算法</t>
         </is>
       </c>
     </row>

</xml_diff>